<commit_message>
Update scripts for OTAA devices
</commit_message>
<xml_diff>
--- a/Arduino/Generic_Simple_Sensor_Node/watermark.xlsx
+++ b/Arduino/Generic_Simple_Sensor_Node/watermark.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cpham/Library/CloudStorage/GoogleDrive-congduc.pham@waziup.org/Mon Drive/Arduino/sketch/00-PRIMA-Intel-Irris/Intelirris_Soil_Sensor/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cpham/Library/CloudStorage/GoogleDrive-congduc.pham@waziup.org/My Drive/Arduino/sketch/00-PEPR-AgriFutur/Generic_Simple_Sensor_Node/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70A053E8-30A8-3C47-9357-FA53031BEB20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{126B0D7D-35BC-F642-BA2A-8C45477D8158}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3180" yWindow="1940" windowWidth="28160" windowHeight="16880" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1240" yWindow="1940" windowWidth="28160" windowHeight="16880" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -78,8 +78,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -167,7 +168,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -183,6 +184,9 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -473,15 +477,15 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="15"/>
+      <c r="B2" s="18"/>
       <c r="C2" t="s">
         <v>9</v>
       </c>
       <c r="D2" s="7">
-        <v>1044</v>
+        <v>2232</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -514,15 +518,15 @@
       </c>
       <c r="D5" s="2">
         <f>ABS(($D$2/1000*23.156-12.736)-(1+0.018*($A5-24)))</f>
-        <v>10.366864</v>
-      </c>
-      <c r="E5" s="2">
+        <v>37.876192000000003</v>
+      </c>
+      <c r="E5" s="15">
         <f>ABS((-3.213*($D$2/1000)-4.093)/(1-0.009733*($D$2/1000)-0.01205*($A5)))</f>
-        <v>11.414668461720485</v>
+        <v>17.57659357549548</v>
       </c>
       <c r="F5" s="2">
         <f>ABS(2.246-5.239*($D$2/1000)*(1+0.018*($A5-24))-0.06756*($D$2/1000)*($D$2/1000)*((1+0.018*($A5-24))*(1+0.018*($A5-24))))</f>
-        <v>3.7019425525458547</v>
+        <v>10.676159447079979</v>
       </c>
       <c r="G5" t="s">
         <v>6</v>
@@ -541,15 +545,15 @@
       </c>
       <c r="D6" s="4">
         <f>ABS(($D$2/1000*23.156-12.736)-(1+0.018*($A6-24)))</f>
-        <v>10.438863999999999</v>
-      </c>
-      <c r="E6" s="4">
+        <v>37.948192000000006</v>
+      </c>
+      <c r="E6" s="16">
         <f>ABS((-3.213*($D$2/1000)-4.093)/(1-0.009733*($D$2/1000)-0.01205*($A6)))</f>
-        <v>10.629403556767031</v>
+        <v>16.347132849554246</v>
       </c>
       <c r="F6" s="4">
         <f>ABS(2.246-5.239*($D$2/1000)*(1+0.018*($A6-24))-0.06756*($D$2/1000)*($D$2/1000)*((1+0.018*($A6-24))*(1+0.018*($A6-24))))</f>
-        <v>3.2971520761600006</v>
+        <v>9.7840200294399988</v>
       </c>
       <c r="G6" t="s">
         <v>7</v>
@@ -557,7 +561,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="11">
-        <v>9</v>
+        <v>17.5</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>5</v>
@@ -568,15 +572,15 @@
       </c>
       <c r="D7" s="6">
         <f>ABS(($D$2/1000*23.156-12.736)-(1+0.018*($A7-24)))</f>
-        <v>10.708863999999998</v>
-      </c>
-      <c r="E7" s="6">
+        <v>38.065192000000003</v>
+      </c>
+      <c r="E7" s="17">
         <f>ABS((-3.213*($D$2/1000)-4.093)/(1-0.009733*($D$2/1000)-0.01205*($A7)))</f>
-        <v>8.4495882400350304</v>
+        <v>14.678657992372761</v>
       </c>
       <c r="F7" s="6">
         <f>ABS(2.246-5.239*($D$2/1000)*(1+0.018*($A7-24))-0.06756*($D$2/1000)*($D$2/1000)*((1+0.018*($A7-24))*(1+0.018*($A7-24))))</f>
-        <v>1.7859873449856642</v>
+        <v>8.3417360930620443</v>
       </c>
       <c r="G7" t="s">
         <v>8</v>

</xml_diff>